<commit_message>
Proposition E17 pour Antoine Latreille (pacte d'associés, T9), sans mention de la loi PACTE à l'oral.
Les pages capsule affichent désormais le script validé ou la proposition éditoriale à la place de la projection générique.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/20260723_Prev_Vid.xlsx
+++ b/data/20260723_Prev_Vid.xlsx
@@ -633,8 +633,8 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>E2 — Passer d’une technologie à un problème à résoudre. Utilisateur, client, bénéficiaire, usage et proposition de valeur. 
-E3 — Poser ou identifier le bon problème avant de chercher la solution. Validation, hypothèses, expérimentation, pivot et apprentissage.</t>
+          <t>E2 — Joël Nguyen : Passer d’une technologie à un problème à résoudre. Utilisateur, client, bénéficiaire, usage et proposition de valeur. 
+E3 — Gregoire Burgé : Poser ou identifier le bon problème avant de chercher la solution. Validation, hypothèses, expérimentation, pivot et apprentissage.</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -644,7 +644,8 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Gregoire Burgé
+          <t>Joël Nguyen
+Gregoire Burgé
 Bernard Yannou</t>
         </is>
       </c>
@@ -1149,7 +1150,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>E22 — Pascal Corbel : Concevoir une collaboration équilibrée. Objectifs partagés, complémentarité, gouvernance, engagement, création et partage de valeur. 
+          <t>E22 — Rémi Waché : Concevoir une collaboration équilibrée. Objectifs partagés, complémentarité, gouvernance, engagement, création et partage de valeur. 
 E23 — Eneli Vino : Sécuriser juridiquement la collaboration. Confidentialité, contrats, connaissances antérieures, résultats nouveaux, PI, publication et sortie du partenariat.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Placer E11bis sur T6 et figer le statut filmé de chaque vidéo expert.
Le concours scientifique est un régime de l’agent, pas un financement ; la colonne Filmé lit désormais tournage.json pour tout le monde.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/20260723_Prev_Vid.xlsx
+++ b/data/20260723_Prev_Vid.xlsx
@@ -823,12 +823,13 @@
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>E10 — Quelle voie de valorisation pour quel projet ? Licence, création, co-développement, partenariat et critères de choix. 
-E11 — Les mécanismes juridiques du transfert. Licence exclusive ou non, cession, contrat de collaboration, copropriété et principes de négociation.</t>
+E11 — Les mécanismes juridiques du transfert. Licence exclusive ou non, cession, contrat de collaboration, copropriété et principes de négociation.
+E11 bis — Soizic Lefeuvre : La loi PACTE et le concours scientifique (optionnel). Régime de l’agent public (loi Allègre 1999 / loi PACTE 2019) : participer à une société qui valorise ses travaux sans quitter l’établissement. Ce n’est pas un concours de financement. Distinct du pacte d’associés (E17).</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>L’apprenant comprend que la création d’entreprise n’est qu’une voie possible. Il sait comparer les grandes options et identifier les questions à traiter avec les professionnels de la valorisation.</t>
+          <t>L’apprenant comprend que la création d’entreprise n’est qu’une voie possible. Il sait comparer les grandes options et identifier les questions à traiter avec les professionnels de la valorisation. En option, s’il choisit la création, il sait que le concours scientifique est un régime de l’agent (temps, parts, fonctions), pas un financement.</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Ajouter l'onglet Monica et le document unique d'arbitrage avec les propositions Clarisse.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/20260723_Prev_Vid.xlsx
+++ b/data/20260723_Prev_Vid.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feuil1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>